<commit_message>
Momskoder steg 2: momskod och leveransdatum på fakturaraderna, momsnummer och undantagstexter på dokumenten, land och momskod på leverantören
Fakturaraderna får sin momskod härledd ur kundens land, momsnummer,
privatperson och omvänd betalningsskyldighet för byggtjänster (ren
salesVatCode i shared), Utfärda vägrar EU-försäljning och omvänd
betalningsskyldighet utan giltigt momsnummer, raderna bär
leveransdatum från kundorderradens senaste leverans, faktura-PDF:en
skriver köparens momsnummer, kodernas texter och Levererad-datum,
e-fakturan skriver omvänd betalningsskyldighet som AE, och leverantören
får land och förvald momskod som leverantörsfakturan ärver.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RSdtiEAvRGDcuA9MaSsvt
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-leverantorer.xlsx
+++ b/apps/web/public/importmallar/importmall-leverantorer.xlsx
@@ -166,11 +166,23 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">Landskod med två bokstäver (t.ex. SE); små bokstäver godtas. Styr leverantörsfakturans förvalda momskod när leverantören saknar egen: SE ger svensk moms, ett annat EU-land omvänd moms på varor och övriga länder varor utanför EU. Tom cell ger SE på en ny leverantör. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">Valutakod med tre bokstäver (SEK, EUR, NOK …); små bokstäver godtas, annat ger ett fel. Nya inköpsorder och nya katalograder (även de som Inköpspriser-importen skapar) får leverantörens valuta; befintliga behåller sin. Tom cell ger SEK för nya leverantörer och lämnar befintliga orörda.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -182,7 +194,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -194,7 +206,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0">
+    <comment ref="Q1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -206,7 +218,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="R1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -218,7 +230,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0">
+    <comment ref="S1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -302,12 +314,13 @@
     <col min="10" max="10" width="15" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1" style="4"/>
     <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1" style="4"/>
-    <col min="14" max="14" width="19" customWidth="1" style="4"/>
-    <col min="15" max="15" width="21" customWidth="1" style="4"/>
-    <col min="16" max="16" width="19" customWidth="1" style="4"/>
-    <col min="17" max="17" width="25" customWidth="1" style="4"/>
-    <col min="18" max="18" width="27" customWidth="1" style="4"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1" style="4"/>
+    <col min="15" max="15" width="19" customWidth="1" style="4"/>
+    <col min="16" max="16" width="21" customWidth="1" style="4"/>
+    <col min="17" max="17" width="19" customWidth="1" style="4"/>
+    <col min="18" max="18" width="25" customWidth="1" style="4"/>
+    <col min="19" max="19" width="27" customWidth="1" style="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -373,30 +386,35 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Land</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Valuta</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Vårt kundnummer</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Betalningsvillkor</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Leveransvillkor</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Leveranssätt/speditör</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Kundnummer hos speditör</t>
         </is>
@@ -743,7 +761,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valuta</t>
+          <t xml:space="preserve">Land</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -753,19 +771,19 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valutakod med tre bokstäver (SEK, EUR, NOK …); små bokstäver godtas, annat ger ett fel. Nya inköpsorder och nya katalograder (även de som Inköpspriser-importen skapar) får leverantörens valuta; befintliga behåller sin. Tom cell ger SEK för nya leverantörer och lämnar befintliga orörda.</t>
+          <t xml:space="preserve">Landskod med två bokstäver (t.ex. SE); små bokstäver godtas. Styr leverantörsfakturans förvalda momskod när leverantören saknar egen: SE ger svensk moms, ett annat EU-land omvänd moms på varor och övriga länder varor utanför EU. Tom cell ger SE på en ny leverantör. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEK</t>
+          <t xml:space="preserve">SE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vårt kundnummer</t>
+          <t xml:space="preserve">Valuta</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -775,19 +793,19 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Det kundnummer leverantören har på oss, max 50 tecken — skrivs ut på förfrågan och inköpsorder. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Valutakod med tre bokstäver (SEK, EUR, NOK …); små bokstäver godtas, annat ger ett fel. Nya inköpsorder och nya katalograder (även de som Inköpspriser-importen skapar) får leverantörens valuta; befintliga behåller sin. Tom cell ger SEK för nya leverantörer och lämnar befintliga orörda.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">K-1234</t>
+          <t xml:space="preserve">SEK</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betalningsvillkor</t>
+          <t xml:space="preserve">Vårt kundnummer</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -797,19 +815,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Betalningsvillkorets kod eller namn i registret (skiftlägesokänsligt), max 100 tecken. Ett okänt värde skapas som nytt villkor; börjar namnet med ett antal dagar (30 dagar netto) blir dagarna villkorets kod och styr förfallodatum på leverantörsfakturor.</t>
+          <t xml:space="preserve">Det kundnummer leverantören har på oss, max 50 tecken — skrivs ut på förfrågan och inköpsorder. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 dagar netto</t>
+          <t xml:space="preserve">K-1234</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leveransvillkor</t>
+          <t xml:space="preserve">Betalningsvillkor</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -819,19 +837,19 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leveransvillkorets kod eller namn i registret (skiftlägesokänsligt), max 100 tecken. Ett okänt värde skapas som nytt villkor.</t>
+          <t xml:space="preserve">Betalningsvillkorets kod eller namn i registret (skiftlägesokänsligt), max 100 tecken. Ett okänt värde skapas som nytt villkor; börjar namnet med ett antal dagar (30 dagar netto) blir dagarna villkorets kod och styr förfallodatum på leverantörsfakturor.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fritt vårt lager</t>
+          <t xml:space="preserve">30 dagar netto</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leveranssätt/speditör</t>
+          <t xml:space="preserve">Leveransvillkor</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -841,32 +859,54 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Speditörens kod eller namn i registret (skiftlägesokänsligt), max 100 tecken. Ett okänt värde skapas som ny speditör.</t>
+          <t xml:space="preserve">Leveransvillkorets kod eller namn i registret (skiftlägesokänsligt), max 100 tecken. Ett okänt värde skapas som nytt villkor.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exempelfrakt</t>
+          <t xml:space="preserve">Fritt vårt lager</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Leveranssätt/speditör</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Speditörens kod eller namn i registret (skiftlägesokänsligt), max 100 tecken. Ett okänt värde skapas som ny speditör.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exempelfrakt</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Kundnummer hos speditör</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nej</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Vårt kundnummer hos leverantörens speditör, max 50 tecken. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">F-98765</t>
         </is>

</xml_diff>